<commit_message>
Add Outlook Revisi module and improve HRIS assisted upload
</commit_message>
<xml_diff>
--- a/config/hris/OAS-K_HRIS_Configuration.xlsx
+++ b/config/hris/OAS-K_HRIS_Configuration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python Project\OfficeAutomationSuite-Karina\config\hris\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A87991-6749-4291-89F9-74446A2F37B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_19D290ACC5F4C1D9AE2162410BB6338EB6E1A265" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -18,13 +18,132 @@
     <sheet name="Browser" sheetId="3" r:id="rId3"/>
     <sheet name="Upload" sheetId="4" r:id="rId4"/>
     <sheet name="Reference" sheetId="5" r:id="rId5"/>
+    <sheet name="Assisted_Steps" sheetId="6" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Assisted_Steps!$A$1:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Upload!$A$1:$C$31</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="196">
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Sequence</t>
+  </si>
+  <si>
+    <t>Step_Name</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Input_Source</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>Wait_After_Seconds</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>run_control_id</t>
+  </si>
+  <si>
+    <t>click_type</t>
+  </si>
+  <si>
+    <t>RUN_CONTROL_ID</t>
+  </si>
+  <si>
+    <t>coordinate</t>
+  </si>
+  <si>
+    <t>Focus Run Control field and type current Run Control ID</t>
+  </si>
+  <si>
+    <t>start_date</t>
+  </si>
+  <si>
+    <t>START_DATE</t>
+  </si>
+  <si>
+    <t>Focus Start Date field and type Start Date</t>
+  </si>
+  <si>
+    <t>end_date</t>
+  </si>
+  <si>
+    <t>END_DATE</t>
+  </si>
+  <si>
+    <t>Focus End Date field and type End Date</t>
+  </si>
+  <si>
+    <t>add_attachment</t>
+  </si>
+  <si>
+    <t>click</t>
+  </si>
+  <si>
+    <t>NONE</t>
+  </si>
+  <si>
+    <t>Click Add Attachment</t>
+  </si>
+  <si>
+    <t>choose_file</t>
+  </si>
+  <si>
+    <t>attach_file</t>
+  </si>
+  <si>
+    <t>TXT_FILE_PATH</t>
+  </si>
+  <si>
+    <t>assisted</t>
+  </si>
+  <si>
+    <t>Attach or choose TXT file for current item</t>
+  </si>
+  <si>
+    <t>upload</t>
+  </si>
+  <si>
+    <t>Click Upload</t>
+  </si>
+  <si>
+    <t>ok_after_upload</t>
+  </si>
+  <si>
+    <t>Click OK after Upload</t>
+  </si>
+  <si>
+    <t>run</t>
+  </si>
+  <si>
+    <t>Click Run</t>
+  </si>
+  <si>
+    <t>ok_after_run</t>
+  </si>
+  <si>
+    <t>Click OK after Run</t>
+  </si>
   <si>
     <t>Parameter</t>
   </si>
@@ -32,9 +151,6 @@
     <t>Value</t>
   </si>
   <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>HRIS_URL</t>
   </si>
   <si>
@@ -83,10 +199,10 @@
     <t>New / Resume. GUI will control this later.</t>
   </si>
   <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Sequence</t>
+    <t>Folder_Upload_Path</t>
+  </si>
+  <si>
+    <t>D:\Python Project\OfficeAutomationSuite-Karina\output\HRIS</t>
   </si>
   <si>
     <t>Workflow</t>
@@ -95,9 +211,6 @@
     <t>Run_Control_ID</t>
   </si>
   <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>001</t>
   </si>
   <si>
@@ -290,6 +403,138 @@
     <t>Folder for Upload_Report, Upload_Process.log, Upload_Summary.json.</t>
   </si>
   <si>
+    <t>Click_Profile_Path</t>
+  </si>
+  <si>
+    <t>config\hris\HRIS_Click_Profile.json</t>
+  </si>
+  <si>
+    <t>Path hasil kalibrasi assisted action</t>
+  </si>
+  <si>
+    <t>Assisted_Mode_Enabled</t>
+  </si>
+  <si>
+    <t>Enable assisted automation mode after upload page opened</t>
+  </si>
+  <si>
+    <t>Manual_Recovery_Enabled</t>
+  </si>
+  <si>
+    <t>Pause and allow operator recovery if step fails</t>
+  </si>
+  <si>
+    <t>Require_Profile_Match</t>
+  </si>
+  <si>
+    <t>Validate screen/browser profile before replay</t>
+  </si>
+  <si>
+    <t>Use_Date_From_Config</t>
+  </si>
+  <si>
+    <t>If TRUE, GUI uses Start_Date and End_Date from config</t>
+  </si>
+  <si>
+    <t>Start_Date</t>
+  </si>
+  <si>
+    <t>03/30/2026</t>
+  </si>
+  <si>
+    <t>Optional default start date for HRIS upload</t>
+  </si>
+  <si>
+    <t>End_Date</t>
+  </si>
+  <si>
+    <t>Optional default end date for HRIS upload</t>
+  </si>
+  <si>
+    <t>Browser_X</t>
+  </si>
+  <si>
+    <t>Fixed Edge window X</t>
+  </si>
+  <si>
+    <t>Browser_Y</t>
+  </si>
+  <si>
+    <t>Fixed Edge window Y</t>
+  </si>
+  <si>
+    <t>Browser_Width</t>
+  </si>
+  <si>
+    <t>Fixed Edge window width</t>
+  </si>
+  <si>
+    <t>Browser_Height</t>
+  </si>
+  <si>
+    <t>Fixed Edge window height</t>
+  </si>
+  <si>
+    <t>Browser_Zoom</t>
+  </si>
+  <si>
+    <t>Expected browser zoom percentage</t>
+  </si>
+  <si>
+    <t>Assisted_Verification_Enabled</t>
+  </si>
+  <si>
+    <t>Verify HRIS submission result after Run and OK</t>
+  </si>
+  <si>
+    <t>Verification_Wait_Seconds</t>
+  </si>
+  <si>
+    <t>Initial wait before reading HRIS result text</t>
+  </si>
+  <si>
+    <t>Verification_Timeout_Seconds</t>
+  </si>
+  <si>
+    <t>Maximum automatic verification time per item</t>
+  </si>
+  <si>
+    <t>Verification_Poll_Seconds</t>
+  </si>
+  <si>
+    <t>Interval between HRIS result checks</t>
+  </si>
+  <si>
+    <t>Verification_Success_Texts</t>
+  </si>
+  <si>
+    <t>Process Instance|Submitted|Queued</t>
+  </si>
+  <si>
+    <t>Pipe-separated HRIS submission success phrases</t>
+  </si>
+  <si>
+    <t>Verification_Failure_Texts</t>
+  </si>
+  <si>
+    <t>Error|Invalid|Failed</t>
+  </si>
+  <si>
+    <t>Pipe-separated HRIS failure phrases</t>
+  </si>
+  <si>
+    <t>Manual_Verification_On_Unknown</t>
+  </si>
+  <si>
+    <t>Ask operator when automatic verification is inconclusive</t>
+  </si>
+  <si>
+    <t>Manual_Verification_On_Error</t>
+  </si>
+  <si>
+    <t>Ask operator when an HRIS error phrase is detected</t>
+  </si>
+  <si>
     <t>Item</t>
   </si>
   <si>
@@ -372,19 +617,13 @@
   </si>
   <si>
     <t>Successful TXT files move to Upload folder. Failed TXT files move to Failed folder. Reports/log/json go to Report/&lt;JOB_ID&gt;.</t>
-  </si>
-  <si>
-    <t>Folder_Upload_Path</t>
-  </si>
-  <si>
-    <t>D:\Python Project\OfficeAutomationSuite-Karina\output\HRIS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -395,13 +634,30 @@
       <color rgb="FFFFFFFF"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -421,7 +677,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -433,11 +689,25 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -486,21 +756,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="HRISUploadTable" displayName="HRISUploadTable" ref="A1:C11">
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Parameter"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Description"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="HRISReferenceTable" displayName="HRISReferenceTable" ref="A1:B14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="HRISReferenceTable" displayName="HRISReferenceTable" ref="A1:B14">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Item"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Rule"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Item"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Rule"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -665,90 +924,90 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="56">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="56" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="B5" s="2">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="B6" s="2">
         <v>30</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="28" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>116</v>
+        <v>56</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>117</v>
+        <v>57</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -787,274 +1046,274 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B3" s="2">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>27</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B6" s="2">
         <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B7" s="2">
         <v>6</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B8" s="2">
         <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>37</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B9" s="2">
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>38</v>
+        <v>74</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>39</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2">
         <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>40</v>
+        <v>76</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>41</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B11" s="2">
         <v>10</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>43</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B12" s="2">
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>46</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B13" s="2">
         <v>2</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>48</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B14" s="2">
         <v>3</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>49</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B15" s="2">
         <v>4</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>50</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="B16" s="2">
         <v>5</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>51</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="4:4">
@@ -2537,68 +2796,68 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>53</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>54</v>
+        <v>90</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>56</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>59</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>61</v>
+        <v>97</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>62</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2622,7 +2881,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -2632,135 +2891,353 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>65</v>
+        <v>101</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>66</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>67</v>
+        <v>103</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>68</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>69</v>
+        <v>105</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>70</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>73</v>
+        <v>109</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>74</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>75</v>
+        <v>111</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>76</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>77</v>
+        <v>113</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>78</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>81</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="2" t="s">
-        <v>82</v>
+        <v>118</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>83</v>
+        <v>119</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>84</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>87</v>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="28" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B19" s="2">
+        <v>0</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B20" s="2">
+        <v>0</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B21" s="2">
+        <v>1200</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B22" s="2">
+        <v>800</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B23" s="2">
+        <v>100</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B25" s="2">
+        <v>1</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B26" s="2">
+        <v>10</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B27" s="2">
+        <v>1</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="28">
+      <c r="A28" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C31" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" sqref="B2:B8" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -2775,114 +3252,114 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>168</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>89</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>90</v>
+        <v>170</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>91</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>92</v>
+        <v>172</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>93</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
-        <v>94</v>
+        <v>174</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>95</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
-        <v>96</v>
+        <v>176</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>97</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
-        <v>98</v>
+        <v>178</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>99</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>101</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
-        <v>102</v>
+        <v>182</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>103</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
-        <v>104</v>
+        <v>184</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>105</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>106</v>
+        <v>186</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>107</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>108</v>
+        <v>188</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>109</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>110</v>
+        <v>190</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>111</v>
+        <v>191</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>112</v>
+        <v>192</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>113</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="28" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>114</v>
+        <v>194</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>115</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -2891,4 +3368,337 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="64" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="24" customHeight="1">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="2">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="2">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2">
+        <v>2</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="2">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="2">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="2">
+        <v>2</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="2">
+        <v>1</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I10" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <conditionalFormatting sqref="A2:I10">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$A2="N"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="5">
+    <dataValidation type="list" sqref="A2:A500" xr:uid="{00000000-0002-0000-0500-000000000000}">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="D2:D500" xr:uid="{00000000-0002-0000-0500-000001000000}">
+      <formula1>"click,click_type,type,press,attach_file,wait,manual_continue"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="E2:E500" xr:uid="{00000000-0002-0000-0500-000002000000}">
+      <formula1>"NONE,RUN_CONTROL_ID,START_DATE,END_DATE,TXT_FILE_PATH"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="F2:F500" xr:uid="{00000000-0002-0000-0500-000003000000}">
+      <formula1>"coordinate,playwright,manual,assisted"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="G2:G500" xr:uid="{00000000-0002-0000-0500-000004000000}">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>